<commit_message>
description added to bulk import
</commit_message>
<xml_diff>
--- a/bulk_product_import_template.xlsx
+++ b/bulk_product_import_template.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="37">
   <si>
     <t xml:space="preserve">Category</t>
   </si>
@@ -79,6 +79,9 @@
     <t xml:space="preserve">Is_live</t>
   </si>
   <si>
+    <t xml:space="preserve">Description</t>
+  </si>
+  <si>
     <t xml:space="preserve">Thamboolam bags</t>
   </si>
   <si>
@@ -98,6 +101,9 @@
   </si>
   <si>
     <t xml:space="preserve">No</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gjgjgjgjhgjgjgjg</t>
   </si>
   <si>
     <t xml:space="preserve">Luxury Carry Bag</t>
@@ -134,7 +140,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -164,6 +170,14 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -207,7 +221,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -217,6 +231,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -416,7 +434,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:S4"/>
+  <dimension ref="A1:T4"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17"/>
@@ -435,6 +453,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="19"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="18" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="17.24"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -495,22 +514,25 @@
       <c r="S1" s="2" t="s">
         <v>18</v>
       </c>
+      <c r="T1" s="3" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>250</v>
@@ -534,16 +556,16 @@
         <v>500</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="O2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="P2" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="Q2" s="1" t="n">
         <v>20</v>
@@ -551,22 +573,25 @@
       <c r="R2" s="1" t="n">
         <v>1</v>
       </c>
+      <c r="T2" s="0" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>19</v>
+      <c r="A3" s="4" t="s">
+        <v>20</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F3" s="1" t="n">
         <v>120</v>
@@ -590,16 +615,16 @@
         <v>250</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="N3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="P3" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="O3" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="P3" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="Q3" s="1" t="n">
         <v>50</v>
@@ -610,19 +635,19 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F4" s="1" t="n">
         <v>80</v>
@@ -646,16 +671,16 @@
         <v>150</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="N4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="P4" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="O4" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="P4" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="Q4" s="1" t="n">
         <v>100</v>

</xml_diff>